<commit_message>
Add Yagyank Chadha U20291582 FY2026-27 YTD capital gains and interest
Extend the satellite-account Schedule FA workbook with Capital Gains and
Schedule OS for FY 2026-27 through 10-Sep-2026 (GOOG and SHOP sales; nil
dividends; credit interest only).

Co-authored-by: caakshay-ux <caakshay-ux@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/clients/Yagyank_Chadha_U20291582/Foreign_Assets_Schedule_FA_Yagyank_Chadha_U20291582_AY2026-27.xlsx
+++ b/clients/Yagyank_Chadha_U20291582/Foreign_Assets_Schedule_FA_Yagyank_Chadha_U20291582_AY2026-27.xlsx
@@ -20,6 +20,8 @@
     <sheet name="FIFO Lots Register" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="CG Summary by Symbol" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Notes for CA" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Capital Gains FY2026-27" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Schedule OS - FY2026-27" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -471,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Table range for VLOOKUP: A4:C26</t>
+          <t>Table range for VLOOKUP: A4:C33</t>
         </is>
       </c>
     </row>
@@ -859,89 +861,249 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FCY→USD cross rates (IBKR 31-Dec-2025 close — edit if using trade-date FX)</t>
+      <c r="A28" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>Units per 1 FCY → USD</t>
+      <c r="A29" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>DKK</t>
-        </is>
+      <c r="A30" s="2" t="n">
+        <v>46202</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>0.15726</v>
+        <v>93.95</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
+      <c r="A31" s="2" t="n">
+        <v>46203</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>1.1746</v>
+        <v>93.95</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>HKD</t>
-        </is>
+      <c r="A32" s="2" t="n">
+        <v>46234</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>0.12849</v>
+        <v>95.2</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
+      <c r="A33" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.0063827</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SGD</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>0.7776049766718507</v>
+        <v>95</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Month-end card — replace with exact SBI card rate if different</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36"/>
+          <t>FCY→USD cross rates (IBKR 31-Dec-2025 close — edit if using trade-date FX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>Units per 1 FCY → USD</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
       <c r="A37" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1.2615</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CNH</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0.14905</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0.14905</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0.15726</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>1.1746</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1.342</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0.12849</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0.0063827</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0.7776049766718507</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>TWD</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0.031725</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Yellow/input cells on CG sheets: Sale/Cost FCY, Comm USD, FX rates. All P&amp;L columns are formulas.</t>
         </is>
@@ -1115,7 +1277,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="G6" s="4" t="n"/>
       <c r="T6" s="4" t="n"/>
@@ -1128,7 +1289,6 @@
       <c r="G8" s="4" t="n"/>
       <c r="T8" s="4" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1254,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1297,7 +1457,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1308,6 +1467,89 @@
         <is>
           <t>Detail P&amp;L with editable FX is on 'Capital Gains FY2025-26' (formula-driven). This summary is a static cross-check.</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>— FY 2026-27 YTD (to 10-Sep-2026) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>STCG INR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>LTCG INR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Total Gain/(Loss) INR</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sale Proceeds USD</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cost USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1222236</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1222236</v>
+      </c>
+      <c r="E7" t="n">
+        <v>40373.86</v>
+      </c>
+      <c r="F7" t="n">
+        <v>29286.46</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>327389</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>327389</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6389.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3309.68</v>
       </c>
     </row>
   </sheetData>
@@ -1321,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1343,7 +1585,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yagyank Chadha — IBKR U20291582 (Individual) — Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED</t>
+          <t>Yagyank Chadha (also spelled Chaddha) — IBKR U20291582 (Individual) — Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED. Satellite / Chaddha_1 account.</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1597,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Real IBKR Activity Statement FY2025-26 (23-May-2025–31-Mar-2026). CY2025 Annual synthesized; YE marks from PortfolioAnalyst CY2025 Open Position Summary.</t>
+          <t>Real IBKR Activity Statement FY2025-26 (23-May-2025–31-Mar-2026). FY2026-27 YTD Activity Statement (01-Apr-2026–10-Sep-2026). CY2025 Annual synthesized; YE marks from PortfolioAnalyst CY2025 Open Position Summary.</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1609,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Opened 23-May-2025 via Internal In from U15172057: SHOP × 84, Fidelity Global Technology LU0099574567 × 511.42, BGF World Financials LU0106831901 × 792.45. FOP/ACATS In GOOG × 105 on 01-Dec-2025.</t>
+          <t>Opened 23-May-2025 via Internal In from U15172057: SHOP × 84, Fidelity Global Technology LU0099574567 × 511.42, BGF World Financials LU0106831901 × 792.45. FOP/ACATS In GOOG × 105 on 01-Dec-2025. FOP In GOOG × 323 on 08-Sep-2026.</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1628,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Capital gains</t>
+          <t>Capital gains FY2025-26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1398,199 +1640,199 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dividends / FTC</t>
+          <t>Capital gains FY2026-27 YTD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GOOG USD 22.05 on 15-Dec-2025 and 16-Mar-2026 (FY total USD 44.10). US withholding 25% (USD 5.51 × 2) — see FTC sheet.</t>
+          <t>Partial (to 10-Sep-2026): taxable sales of GOOG × 105 (12-May-2026) and SHOP × 44 (Jul–Aug 2026). Acquisition dates = inbound transfer dates (confirm original buys at U15172057 / prior broker for LTCG — workbook uses transfer dates → STCG if &lt;730 days).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cost / acquisition dates</t>
+          <t>Dividends / FTC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cost basis from IBKR Open Positions carryover. Acquisition dates = inbound transfer dates. Confirm original buy dates at U15172057 / prior broker for LTCG on future sales (SHOP/funds originally FOP into U15172057 in Sep-2024).</t>
+          <t>FY2025-26: GOOG USD 22.05 on 15-Dec-2025 and 16-Mar-2026 (FY total USD 44.10); US withholding 25% (USD 5.51 × 2) — see FTC sheet. FY2026-27 YTD: nil dividends; interest only (USD credit interest).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Assessee</t>
+          <t>Cost / acquisition dates</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yagyank Chadha</t>
+          <t>Cost basis from IBKR Open Positions carryover. Acquisition dates = inbound transfer dates. Confirm original buy dates at U15172057 / prior broker for LTCG on future sales (SHOP/funds originally FOP into U15172057 in Sep-2024).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Account</t>
+          <t>Assessee</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U20291582 — Interactive Brokers LLC (Advisor Client; Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED)</t>
+          <t>Yagyank Chadha</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Customer type</t>
+          <t>Account</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>U20291582 — Interactive Brokers LLC (Advisor Client; Advisor: MATCAP WEALTH ADVISORS PRIVATE LIMITED)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Base currency</t>
+          <t>Customer type</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Individual</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Account funded</t>
+          <t>Base currency</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>First deposit n/a (inception statement)</t>
+          <t>USD</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Schedule FA period</t>
+          <t>Account funded</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Calendar Year 2025 (01-Jan-2025 to 31-Dec-2025) — for ITR AY 2026-27</t>
+          <t>First deposit n/a (inception statement)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Income / CG period</t>
+          <t>Schedule FA period</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FY 2025-26 (01-Apr-2025 to 31-Mar-2026); also FY 2024-25 sheet for prior year</t>
+          <t>Calendar Year 2025 (01-Jan-2025 to 31-Dec-2025) — for ITR AY 2026-27</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Source data</t>
+          <t>Income / CG period</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IBKR Activity Statements: Inception FY2024-25 + Annual CY2025 + Fiscal FY2025-26</t>
+          <t>FY 2025-26 (01-Apr-2025 to 31-Mar-2026); also FY 2024-25 sheet for prior year</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FIFO method</t>
+          <t>Source data</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Actual buy dates &amp; IBKR Basis from inception replay; splits (LRCX 10:1, NFLX 10:1) applied</t>
+          <t>IBKR Activity Statements: Inception FY2024-25 + Annual CY2025 + Fiscal FY2025-26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CG reconciliation</t>
+          <t>FIFO method</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sheets 'Capital Gains FY2025-26' / 'FY2024-25' are formula-driven — yellow cells editable; Gain = Sale INR − Comm INR − Cost INR</t>
+          <t>Actual buy dates &amp; IBKR Basis from inception replay; splits (LRCX 10:1, NFLX 10:1) applied</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FX Lookup</t>
+          <t>CG reconciliation</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Editable SBI TT USD/INR &amp; EUR/INR month-end rates + FCY→USD cross rates</t>
+          <t>Sheets 'Capital Gains FY2025-26' / 'FY2024-25' are formula-driven — yellow cells editable; Gain = Sale INR − Comm INR − Cost INR</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Starting NAV CY2025</t>
+          <t>FX Lookup</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>USD 0.00</t>
+          <t>Editable SBI TT USD/INR &amp; EUR/INR month-end rates + FCY→USD cross rates</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ending NAV CY2025</t>
+          <t>Starting NAV CY2025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>USD 156,356.25</t>
+          <t>USD 0.00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Deposits CY2025</t>
+          <t>Ending NAV CY2025</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>USD 0.00</t>
+          <t>USD 156,356.25</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deposits since inception (to 31-Mar-2025)</t>
+          <t>Deposits CY2025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1602,67 +1844,67 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dividends CY2025</t>
+          <t>Deposits since inception (to 31-Mar-2025)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>USD 22.05 / INR 1,961 (Rule 115)</t>
+          <t>USD 0.00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Interest CY2025</t>
+          <t>Dividends CY2025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>USD 0.00 / INR 0 (Rule 115)</t>
+          <t>USD 22.05 / INR 1,961 (Rule 115)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dividends FY2025-26</t>
+          <t>Interest CY2025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>USD 44.10 / INR 3,958</t>
+          <t>USD 0.00 / INR 0 (Rule 115)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Interest FY2025-26</t>
+          <t>Dividends FY2025-26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>USD 0.00 / INR 0</t>
+          <t>USD 44.10 / INR 3,958</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>STCG FY2025-26 (INR)</t>
+          <t>Interest FY2025-26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>USD 0.00 / INR 0</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LTCG FY2025-26 (INR)</t>
+          <t>STCG FY2025-26 (INR)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1674,7 +1916,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>STCG FY2024-25 (INR)</t>
+          <t>LTCG FY2025-26 (INR)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1686,7 +1928,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LTCG FY2024-25 (INR)</t>
+          <t>STCG FY2024-25 (INR)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1698,133 +1940,1067 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>A1 Foreign Bank/Depository</t>
+          <t>LTCG FY2024-25 (INR)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Generally N/A separately — multi-currency cash sits inside IBKR custodial account (A2)</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>A2 Custodial Account</t>
+          <t>A1 Foreign Bank/Depository</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Applicable — see sheet; opening: 2025-05-23 (Internal In from U15172057)</t>
+          <t>Generally N/A separately — multi-currency cash sits inside IBKR custodial account (A2)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>A3 Equity &amp; Debt Interest</t>
+          <t>A2 Custodial Account</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Applicable — 4 FIFO lot lines (one row per acquisition lot; sold lots match Capital Gains)</t>
+          <t>Applicable — see sheet; opening: 2025-05-23 (Internal In from U15172057)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>A3 Col C (Name of entity)</t>
+          <t>A3 Equity &amp; Debt Interest</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Symbol only (e.g. NOVd, AAPL). Legal name / address remain in Address &amp; Nature columns.</t>
+          <t>Applicable — 4 FIFO lot lines (one row per acquisition lot; sold lots match Capital Gains)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>A3 vs CG</t>
+          <t>A3 Col C (Name of entity)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
+          <t>Symbol only (e.g. NOVd, AAPL). Legal name / address remain in Address &amp; Nature columns.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ADR country practice</t>
+          <t>A3 vs CG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
+          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CPNG</t>
+          <t>ADR country practice</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
+          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NFLX split</t>
+          <t>CPNG</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
+          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LRCX split</t>
+          <t>NFLX split</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
+          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HYU</t>
+          <t>LRCX split</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>HYU</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>Action required</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>1) Confirm exact SBI TT Buy card rates; 2) Obtain PortfolioAnalyst for true peak NAV; 3) Map withholding to Schedule FSI/TR under DTAA.</t>
         </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>FY 2026-27 YTD (01-Apr-2026 to 10-Sep-2026) — partial statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Dividends FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>USD 0.00 / INR 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Interest FY2026-27 YTD</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>USD 126.95 / INR 11,961</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>STCG FY2026-27 YTD (INR)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1,549,625</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LTCG FY2026-27 YTD (INR)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FY2026-27 coverage</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Activity Statement ends 10-Sep-2026 — not full FY. Obtain statement to 31-Mar-2027 for complete year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GOOG FOP 08-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>FOP In GOOG × 323 after May sale — held at period end; not taxable CG. Confirm original buy dates for LTCG on future sales.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Capital gains — FY 2026-27 YTD (01-Apr-2026 to 10-Sep-2026). Partial year — statement ends 10-Sep-2026. FIFO. Yellow cells editable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RECONCILIATION SHEET (formula-driven). Gain/(Loss) INR = Sale INR − Comm INR − Cost INR. Holding &gt;730 → LTCG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F=E-D | G=IF(F&gt;730,"LTCG","STCG") | L=H*K | M=I*K | Q=L*N | R=J*P | S=M*O | T=Q-R-S</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>CCY</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Acquisition Date</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Date</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Holding Days</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Proceeds (FCY)</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Cost Basis (FCY)</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Comm (USD)</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>FCY→USD Rate</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>Sale Proceeds (USD)</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Cost (USD)</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Sale FX Rate</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>Cost FX Rate</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>Comm USD/INR Rate</t>
+        </is>
+      </c>
+      <c r="Q4" s="1" t="inlineStr">
+        <is>
+          <t>Sale (INR)</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>Comm (INR)</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>Cost (INR)</t>
+        </is>
+      </c>
+      <c r="T4" s="1" t="inlineStr">
+        <is>
+          <t>Gain/(Loss) INR</t>
+        </is>
+      </c>
+      <c r="U4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>105</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="F5">
+        <f>E5-D5</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IF(F5&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>40373.86</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>29286.46</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <f>H5*K5</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>I5*K5</f>
+        <v/>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>88.95</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="Q5">
+        <f>L5*N5</f>
+        <v/>
+      </c>
+      <c r="R5">
+        <f>J5*P5</f>
+        <v/>
+      </c>
+      <c r="S5">
+        <f>M5*O5</f>
+        <v/>
+      </c>
+      <c r="T5">
+        <f>Q5-R5-S5</f>
+        <v/>
+      </c>
+      <c r="U5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>45800</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F6">
+        <f>E6-D6</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IF(F6&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>617</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>376.1</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <f>H6*K6</f>
+        <v/>
+      </c>
+      <c r="M6">
+        <f>I6*K6</f>
+        <v/>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="Q6">
+        <f>L6*N6</f>
+        <v/>
+      </c>
+      <c r="R6">
+        <f>J6*P6</f>
+        <v/>
+      </c>
+      <c r="S6">
+        <f>M6*O6</f>
+        <v/>
+      </c>
+      <c r="T6">
+        <f>Q6-R6-S6</f>
+        <v/>
+      </c>
+      <c r="U6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>45800</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="F7">
+        <f>E7-D7</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IF(F7&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>634.5</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>376.1</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <f>H7*K7</f>
+        <v/>
+      </c>
+      <c r="M7">
+        <f>I7*K7</f>
+        <v/>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="Q7">
+        <f>L7*N7</f>
+        <v/>
+      </c>
+      <c r="R7">
+        <f>J7*P7</f>
+        <v/>
+      </c>
+      <c r="S7">
+        <f>M7*O7</f>
+        <v/>
+      </c>
+      <c r="T7">
+        <f>Q7-R7-S7</f>
+        <v/>
+      </c>
+      <c r="U7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>45800</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="F8">
+        <f>E8-D8</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IF(F8&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>3010</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>1504.4</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <f>H8*K8</f>
+        <v/>
+      </c>
+      <c r="M8">
+        <f>I8*K8</f>
+        <v/>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="Q8">
+        <f>L8*N8</f>
+        <v/>
+      </c>
+      <c r="R8">
+        <f>J8*P8</f>
+        <v/>
+      </c>
+      <c r="S8">
+        <f>M8*O8</f>
+        <v/>
+      </c>
+      <c r="T8">
+        <f>Q8-R8-S8</f>
+        <v/>
+      </c>
+      <c r="U8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>45800</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="F9">
+        <f>E9-D9</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(F9&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>526.54</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <f>H9*K9</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>I9*K9</f>
+        <v/>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="Q9">
+        <f>L9*N9</f>
+        <v/>
+      </c>
+      <c r="R9">
+        <f>J9*P9</f>
+        <v/>
+      </c>
+      <c r="S9">
+        <f>M9*O9</f>
+        <v/>
+      </c>
+      <c r="T9">
+        <f>Q9-R9-S9</f>
+        <v/>
+      </c>
+      <c r="U9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>45800</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F10">
+        <f>E10-D10</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IF(F10&gt;730,"LTCG","STCG")</f>
+        <v/>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>1078</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>526.54</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <f>H10*K10</f>
+        <v/>
+      </c>
+      <c r="M10">
+        <f>I10*K10</f>
+        <v/>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="Q10">
+        <f>L10*N10</f>
+        <v/>
+      </c>
+      <c r="R10">
+        <f>J10*P10</f>
+        <v/>
+      </c>
+      <c r="S10">
+        <f>M10*O10</f>
+        <v/>
+      </c>
+      <c r="T10">
+        <f>Q10-R10-S10</f>
+        <v/>
+      </c>
+      <c r="U10" t="inlineStr"/>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL STCG (INR)</t>
+        </is>
+      </c>
+      <c r="T12" s="4">
+        <f>SUMIF(G5:G10,"STCG",T5:T10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL LTCG (INR)</t>
+        </is>
+      </c>
+      <c r="T13" s="4">
+        <f>SUMIF(G5:G10,"LTCG",T5:T10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL CG (INR)</t>
+        </is>
+      </c>
+      <c r="T14" s="4">
+        <f>T12+T13</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A3:U3"/>
+    <mergeCell ref="A2:U2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Interest &amp; Dividend income — FY 2026-27 YTD (01-Apr-2026 to 10-Sep-2026). Partial — full year needs statement through 31-Mar-2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (FCY)</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (USD)</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>USD/INR (Rule 115)</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Amount (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>— INTEREST —</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>USD Credit Interest for May-2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>50.16</v>
+      </c>
+      <c r="E4" t="n">
+        <v>50.16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4745</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USD Credit Interest for Jun-2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>75.88</v>
+      </c>
+      <c r="E5" t="n">
+        <v>75.88</v>
+      </c>
+      <c r="F5" t="n">
+        <v>93.95</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7129</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USD Credit Interest for Jul-2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F6" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TOTAL INTEREST</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>126.95</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11961</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>— DIVIDENDS —</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TOTAL DIVIDENDS</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1924,7 +3100,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="n">
         <v>1</v>
@@ -2163,7 +3338,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="G10" t="inlineStr">
         <is>
@@ -2538,7 +3712,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -2687,7 +3860,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -2836,7 +4008,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -2905,7 +4076,6 @@
         <v>1961</v>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3035,7 +4205,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -3170,7 +4339,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -3579,7 +4747,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="G6" s="4" t="n"/>
       <c r="T6" s="4" t="n"/>
@@ -3592,7 +4759,6 @@
       <c r="G8" s="4" t="n"/>
       <c r="T8" s="4" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>

</xml_diff>